<commit_message>
getting experiment topo and shear stress
</commit_message>
<xml_diff>
--- a/Topography/LaJara_TopoSurvey/LaJara_XS_Topography .xlsx
+++ b/Topography/LaJara_TopoSurvey/LaJara_XS_Topography .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\La_Jara\Topography\LaJara_TopoSurvey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E028F04-81A2-4210-B36D-9C7787A723AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C37771-0D96-4BA5-A144-72D5CDDBBEB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="195" windowWidth="25440" windowHeight="15390" tabRatio="804" firstSheet="9" activeTab="23" xr2:uid="{24083E57-F3BF-4A8D-A2E4-8E86074BFB86}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" tabRatio="804" firstSheet="9" activeTab="23" xr2:uid="{24083E57-F3BF-4A8D-A2E4-8E86074BFB86}"/>
   </bookViews>
   <sheets>
     <sheet name="Piezo 1" sheetId="1" r:id="rId1"/>
@@ -887,7 +887,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-AR"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1356,6 +1356,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1363,7 +1364,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1846,6 +1846,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1853,7 +1854,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2467,6 +2467,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2474,7 +2475,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2945,6 +2945,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2952,7 +2953,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3587,6 +3587,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3594,7 +3595,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4160,6 +4160,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4167,7 +4168,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4826,6 +4826,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4833,7 +4834,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5483,6 +5483,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5490,7 +5491,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5937,6 +5937,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5944,7 +5945,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6401,6 +6401,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6408,7 +6409,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7127,6 +7127,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7134,7 +7135,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7886,6 +7886,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7893,7 +7894,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8527,6 +8527,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8534,7 +8535,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8999,6 +8999,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9006,7 +9007,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9485,6 +9485,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9492,7 +9493,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10064,6 +10064,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10071,7 +10072,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10832,6 +10832,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10839,7 +10840,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -31756,7 +31756,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="1"/>
       <c r="G4" s="2">
-        <f t="shared" ref="G4:G29" si="0">$F$2-C4</f>
+        <f>$F$2-C4</f>
         <v>2737.8500000000004</v>
       </c>
     </row>
@@ -31772,7 +31772,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G4:G29" si="0">$F$2-C5</f>
         <v>2737.59</v>
       </c>
     </row>

</xml_diff>